<commit_message>
Biblioteca actualizada: 121 libros (2026-09-06 19:14)
</commit_message>
<xml_diff>
--- a/LIBRARY.xlsx
+++ b/LIBRARY.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="45" windowWidth="27315" windowHeight="12090"/>
+    <workbookView xWindow="120" yWindow="45" windowWidth="27315" windowHeight="12090" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SCIENCE-FICTION" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,23 @@
     <author>Marcos</author>
   </authors>
   <commentList>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>M: mostaza
+T: Teja
+C: caramelo
+V: Amarilloverdoso</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B84" authorId="0">
       <text>
         <r>
@@ -56,8 +73,42 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Marcos</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>A: Azul P: Morado Q:Aguamarina G:Verde</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="323">
   <si>
     <t>AUTOR</t>
   </si>
@@ -1005,13 +1056,34 @@
   </si>
   <si>
     <t>DATOS</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>G</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1059,6 +1131,19 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1140,7 +1225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1288,6 +1373,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1691,7 +1779,9 @@
         <v>7</v>
       </c>
       <c r="I3" s="43"/>
-      <c r="J3" s="47"/>
+      <c r="J3" s="47" t="s">
+        <v>316</v>
+      </c>
       <c r="K3" s="4"/>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1714,7 +1804,9 @@
         <v>7</v>
       </c>
       <c r="I4" s="43"/>
-      <c r="J4" s="47"/>
+      <c r="J4" s="47" t="s">
+        <v>316</v>
+      </c>
       <c r="K4" s="4"/>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1737,7 +1829,9 @@
         <v>7</v>
       </c>
       <c r="I5" s="43"/>
-      <c r="J5" s="47"/>
+      <c r="J5" s="47" t="s">
+        <v>316</v>
+      </c>
       <c r="K5" s="4"/>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1760,7 +1854,9 @@
         <v>7</v>
       </c>
       <c r="I6" s="43"/>
-      <c r="J6" s="47"/>
+      <c r="J6" s="47" t="s">
+        <v>316</v>
+      </c>
       <c r="K6" s="4"/>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1783,7 +1879,9 @@
         <v>38</v>
       </c>
       <c r="I7" s="43"/>
-      <c r="J7" s="47"/>
+      <c r="J7" s="47" t="s">
+        <v>316</v>
+      </c>
       <c r="K7" s="4"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2546,7 +2644,9 @@
       <c r="I40" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="J40" s="48"/>
+      <c r="J40" s="48" t="s">
+        <v>317</v>
+      </c>
       <c r="K40" s="4"/>
     </row>
     <row r="41" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2571,7 +2671,9 @@
       <c r="I41" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="J41" s="47"/>
+      <c r="J41" s="47" t="s">
+        <v>317</v>
+      </c>
       <c r="K41" s="4"/>
     </row>
     <row r="42" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2596,7 +2698,9 @@
       <c r="I42" s="43" t="s">
         <v>24</v>
       </c>
-      <c r="J42" s="47"/>
+      <c r="J42" s="47" t="s">
+        <v>317</v>
+      </c>
       <c r="K42" s="4"/>
     </row>
     <row r="43" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2621,7 +2725,9 @@
       <c r="I43" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="J43" s="47"/>
+      <c r="J43" s="47" t="s">
+        <v>317</v>
+      </c>
       <c r="K43" s="4"/>
     </row>
     <row r="44" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2646,7 +2752,9 @@
       <c r="I44" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="J44" s="47"/>
+      <c r="J44" s="47" t="s">
+        <v>317</v>
+      </c>
       <c r="K44" s="4"/>
     </row>
     <row r="45" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3233,7 +3341,9 @@
         <v>7</v>
       </c>
       <c r="I69" s="45"/>
-      <c r="J69" s="49"/>
+      <c r="J69" s="49" t="s">
+        <v>318</v>
+      </c>
       <c r="K69" s="4"/>
     </row>
     <row r="70" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3258,7 +3368,9 @@
         <v>7</v>
       </c>
       <c r="I70" s="45"/>
-      <c r="J70" s="49"/>
+      <c r="J70" s="49" t="s">
+        <v>318</v>
+      </c>
       <c r="K70" s="4"/>
     </row>
     <row r="71" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3283,7 +3395,9 @@
         <v>7</v>
       </c>
       <c r="I71" s="45"/>
-      <c r="J71" s="49"/>
+      <c r="J71" s="49" t="s">
+        <v>318</v>
+      </c>
       <c r="K71" s="4"/>
     </row>
     <row r="72" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -3877,7 +3991,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3930,7 +4044,9 @@
       <c r="F2" s="38" t="s">
         <v>267</v>
       </c>
-      <c r="G2" s="40"/>
+      <c r="G2" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="40" t="s">
@@ -3949,7 +4065,9 @@
       <c r="F3" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="G3" s="42"/>
+      <c r="G3" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="40" t="s">
@@ -3968,7 +4086,9 @@
       <c r="F4" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="G4" s="42"/>
+      <c r="G4" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="40" t="s">
@@ -3989,7 +4109,9 @@
       <c r="F5" s="35" t="s">
         <v>253</v>
       </c>
-      <c r="G5" s="41"/>
+      <c r="G5" s="50" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="40" t="s">
@@ -4008,7 +4130,9 @@
       <c r="F6" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="G6" s="42"/>
+      <c r="G6" s="42" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="7" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="40" t="s">
@@ -4025,7 +4149,9 @@
       <c r="F7" s="38" t="s">
         <v>280</v>
       </c>
-      <c r="G7" s="40"/>
+      <c r="G7" s="42" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
@@ -4044,7 +4170,9 @@
       <c r="F8" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="G8" s="40"/>
+      <c r="G8" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="40" t="s">
@@ -4063,7 +4191,9 @@
       <c r="F9" s="38" t="s">
         <v>198</v>
       </c>
-      <c r="G9" s="42"/>
+      <c r="G9" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="40" t="s">
@@ -4082,7 +4212,9 @@
       <c r="F10" s="35" t="s">
         <v>304</v>
       </c>
-      <c r="G10" s="40"/>
+      <c r="G10" s="42" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="11" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="40" t="s">
@@ -4101,7 +4233,9 @@
       <c r="F11" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="40"/>
+      <c r="G11" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="40" t="s">
@@ -4118,7 +4252,9 @@
       <c r="F12" s="38" t="s">
         <v>244</v>
       </c>
-      <c r="G12" s="40"/>
+      <c r="G12" s="42" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="13" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="40" t="s">
@@ -4135,7 +4271,9 @@
       <c r="F13" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="G13" s="42"/>
+      <c r="G13" s="42" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="40" t="s">
@@ -4154,7 +4292,9 @@
       <c r="F14" s="35" t="s">
         <v>203</v>
       </c>
-      <c r="G14" s="42"/>
+      <c r="G14" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="41" t="s">
@@ -4173,7 +4313,7 @@
       <c r="F15" s="38" t="s">
         <v>301</v>
       </c>
-      <c r="G15" s="40"/>
+      <c r="G15" s="42"/>
     </row>
     <row r="16" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="40" t="s">
@@ -4209,7 +4349,7 @@
       <c r="F17" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="G17" s="40"/>
+      <c r="G17" s="42"/>
     </row>
     <row r="18" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="40" t="s">
@@ -4228,7 +4368,9 @@
       <c r="F18" s="38" t="s">
         <v>258</v>
       </c>
-      <c r="G18" s="40"/>
+      <c r="G18" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="19" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="40" t="s">
@@ -4247,7 +4389,7 @@
       <c r="F19" s="38" t="s">
         <v>308</v>
       </c>
-      <c r="G19" s="40"/>
+      <c r="G19" s="42"/>
     </row>
     <row r="20" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="40" t="s">
@@ -4266,7 +4408,7 @@
       <c r="F20" s="35" t="s">
         <v>231</v>
       </c>
-      <c r="G20" s="40"/>
+      <c r="G20" s="42"/>
     </row>
     <row r="21" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="40" t="s">
@@ -4285,7 +4427,7 @@
       <c r="F21" s="38" t="s">
         <v>235</v>
       </c>
-      <c r="G21" s="40"/>
+      <c r="G21" s="42"/>
     </row>
     <row r="22" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="40" t="s">
@@ -4304,7 +4446,9 @@
       <c r="F22" s="35" t="s">
         <v>272</v>
       </c>
-      <c r="G22" s="40"/>
+      <c r="G22" s="42" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="23" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="40" t="s">
@@ -4323,7 +4467,9 @@
       <c r="F23" s="38" t="s">
         <v>217</v>
       </c>
-      <c r="G23" s="42"/>
+      <c r="G23" s="42" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="24" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="40" t="s">
@@ -4342,7 +4488,9 @@
       <c r="F24" s="38" t="s">
         <v>249</v>
       </c>
-      <c r="G24" s="40"/>
+      <c r="G24" s="42" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="25" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="40" t="s">
@@ -4380,7 +4528,9 @@
       <c r="F26" s="38" t="s">
         <v>290</v>
       </c>
-      <c r="G26" s="40"/>
+      <c r="G26" s="42" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="27" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="40" t="s">
@@ -4399,7 +4549,9 @@
       <c r="F27" s="35" t="s">
         <v>295</v>
       </c>
-      <c r="G27" s="40"/>
+      <c r="G27" s="42" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="28" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="40" t="s">
@@ -4418,7 +4570,7 @@
       <c r="F28" s="38" t="s">
         <v>298</v>
       </c>
-      <c r="G28" s="40"/>
+      <c r="G28" s="42"/>
     </row>
     <row r="29" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="40" t="s">
@@ -4437,7 +4589,7 @@
       <c r="F29" s="35" t="s">
         <v>285</v>
       </c>
-      <c r="G29" s="40"/>
+      <c r="G29" s="42"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G29"/>
@@ -4448,5 +4600,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>